<commit_message>
feat(app): Q&A and admin inquiry reply, v2.3.3
Split inquiry into Q&A tabs with history and admin reply flow. Add Admin alarm routing, replyContent, attachment policy, performance tweaks, and bump version to 2.3.3.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/nrm-github-data-fields.xlsx
+++ b/data/nrm-github-data-fields.xlsx
@@ -499,7 +499,7 @@
         <v>선택</v>
       </c>
       <c r="D9" t="str">
-        <v>비어 있으면 전체 사용자에게 표시. 값이 있으면 해당 시리얼(전화번호) 사용자만 표시</v>
+        <v>비어 있으면 전체 사용자에게 표시. 일반 값이면 해당 SerialNo 사용자만 표시. "Admin"은 관리자 전용(문의 알림 등) — versionInfoAdminBuild 또는 userList isAdmin=true 앱만 수신</v>
       </c>
     </row>
     <row r="10">
@@ -650,7 +650,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -782,28 +782,42 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
+        <v>replyContent</v>
+      </c>
+      <c r="B12" t="str">
+        <v>string</v>
+      </c>
+      <c r="C12" t="str">
+        <v>선택</v>
+      </c>
+      <c r="D12" t="str">
+        <v>관리자 답변 본문. 줄바꿈 포함 가능. 미답변 시 빈 문자열</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
         <v>Createddate</v>
       </c>
-      <c r="B12" t="str">
-        <v>string</v>
-      </c>
-      <c r="C12" t="str">
-        <v>필수</v>
-      </c>
-      <c r="D12" t="str">
+      <c r="B13" t="str">
+        <v>string</v>
+      </c>
+      <c r="C13" t="str">
+        <v>필수</v>
+      </c>
+      <c r="D13" t="str">
         <v>등록 시각. 형식: YYYY-MM-DD HH:mm:ss.SSS</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D13"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -947,9 +961,23 @@
         <v>마지막 앱 실행 시각. 형식: YYYY-MM-DD HH:mm:ss.SSS. 미등록 시 null</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>isAdmin</v>
+      </c>
+      <c r="B13" t="str">
+        <v>boolean</v>
+      </c>
+      <c r="C13" t="str">
+        <v>선택</v>
+      </c>
+      <c r="D13" t="str">
+        <v>true면 해당 커스텀 APK가 관리자 권한(Admin SerialNo 알람 수신 등). 기본 admin APK는 versionInfoAdminBuild로 별도 처리</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(app): 관리자·문의·다운로드 개선 및 userList isAdmin 정리, v2.3.7
- GitHub raw JSON 공통 fetch·캐시 버스터, 관리자 사용자 picker/검색 UI

- 문의 첨부 다운로드·알림·로깅 UI 개선, userList isAdmin 필드 제거

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/nrm-github-data-fields.xlsx
+++ b/data/nrm-github-data-fields.xlsx
@@ -499,7 +499,7 @@
         <v>선택</v>
       </c>
       <c r="D9" t="str">
-        <v>비어 있으면 전체 사용자에게 표시. 일반 값이면 해당 SerialNo 사용자만 표시. "Admin"은 관리자 전용(문의 알림 등) — versionInfoAdminBuild 또는 userList isAdmin=true 앱만 수신</v>
+        <v>비어 있으면 SerialNo가 설정된 모든 APK 사용자에게 표시. 값이 있으면 해당 SerialNo APK만 표시. APK SerialNo가 비어 있으면 알림 수집 안 함. "Admin"은 관리자 APK(SerialNo=Admin) 전용</v>
       </c>
     </row>
     <row r="10">
@@ -817,7 +817,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -961,23 +961,9 @@
         <v>마지막 앱 실행 시각. 형식: YYYY-MM-DD HH:mm:ss.SSS. 미등록 시 null</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>isAdmin</v>
-      </c>
-      <c r="B13" t="str">
-        <v>boolean</v>
-      </c>
-      <c r="C13" t="str">
-        <v>선택</v>
-      </c>
-      <c r="D13" t="str">
-        <v>true면 해당 커스텀 APK가 관리자 권한(Admin SerialNo 알람 수신 등). 기본 admin APK는 versionInfoAdminBuild로 별도 처리</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>